<commit_message>
lm, glm, polr models updated
</commit_message>
<xml_diff>
--- a/sharing dataset.xlsx
+++ b/sharing dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pietr\Desktop\Statistical-Inference-Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5698D083-5787-49DE-B209-745C623A14C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{469F3BC7-65ED-4407-8E76-7B5F9FD226DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -467,6 +467,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P519"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" t="s">

</xml_diff>